<commit_message>
addi: set the template's UK DRI defaults for creator, owners, licence and accessRights
Four cells edited in the shipped workbook, making the institutional defaults the
template's own values rather than placeholders:

  catalogue!B4  creator       CREATOR -> UK Dementia Research Institute
  catalogue!B6  license       CC BY 3.0 -> CC BY-NC 4.0
  catalogue!B10 accessRights  GEO/ArrayExpress -> non-commercial use
  workspace_settings!C3 dataset owners  UK DRI PIs -> UK Dementia Research Institute

This is what DESIGN.md and the skill now describe: creator / contactPoint /
dataset owners fall back to these values with a WARN, and accessRights keeps
'non-commercial use'. addi reads them from the template at runtime
(Template.shipped_value), so the docs and the WARN messages track this file.

Dropdowns are intact — 39 zip parts, all 8 x14 data-validations over unchanged
Catalogue_Data ranges, hidden vocab sheet unchanged.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/addi/templates/template_UK_DRI_FAIR_Metadata_w_ExtendedCatalogue_V1.2..xlsx
+++ b/addi/templates/template_UK_DRI_FAIR_Metadata_w_ExtendedCatalogue_V1.2..xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikolaihecker/ukdri/addi/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikolaihecker/ukdri/claude/informatics_data_skills/addi/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15840441-28CC-2E48-B4D2-DBCE7A2EBF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{415EC6A1-D892-854A-92BE-63F02D652580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" tabRatio="910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" tabRatio="910" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="7" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="725">
   <si>
     <t>PLEASE READ CAREFULLY BEFORE FILLING IN THIS TEMPLATE</t>
   </si>
@@ -2349,9 +2349,6 @@
     <t>dataset owners</t>
   </si>
   <si>
-    <t>UK DRI PIs</t>
-  </si>
-  <si>
     <t>geography restrictions</t>
   </si>
   <si>
@@ -2376,9 +2373,6 @@
     <t>license</t>
   </si>
   <si>
-    <t>https://creativecommons.org/licenses/by/3.0/</t>
-  </si>
-  <si>
     <t>versionInfo</t>
   </si>
   <si>
@@ -2391,9 +2385,6 @@
     <t>accessRights</t>
   </si>
   <si>
-    <t>GEO/ArrayExpress</t>
-  </si>
-  <si>
     <t>publisher_name</t>
   </si>
   <si>
@@ -2766,13 +2757,16 @@
     <t>DESCRIPTION</t>
   </si>
   <si>
-    <t>CREATOR</t>
-  </si>
-  <si>
     <t>LIST KEYWORDS</t>
   </si>
   <si>
     <t>IDENTETIFIER</t>
+  </si>
+  <si>
+    <t>https://creativecommons.org/licenses/by-nc/4.0/deed.en</t>
+  </si>
+  <si>
+    <t>non-commercial use</t>
   </si>
 </sst>
 </file>
@@ -2916,7 +2910,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -3149,15 +3143,15 @@
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6736,17 +6730,17 @@
         <v>583</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>584</v>
       </c>
-      <c r="C3" t="s">
-        <v>585</v>
+      <c r="C3" s="4" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C4" t="s">
         <v>583</v>
@@ -6754,15 +6748,15 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C6" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
   </sheetData>
@@ -6807,95 +6801,95 @@
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>724</v>
+        <v>639</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>591</v>
       </c>
-      <c r="B5" s="5" t="s">
+    </row>
+    <row r="6" spans="1:2" s="4" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
         <v>592</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>593</v>
-      </c>
       <c r="B6" s="5" t="s">
-        <v>594</v>
+        <v>723</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="B10" s="51" t="s">
-        <v>599</v>
+        <v>596</v>
+      </c>
+      <c r="B10" s="55" t="s">
+        <v>724</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
     </row>
   </sheetData>
@@ -6928,24 +6922,24 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="53" t="s">
-        <v>608</v>
-      </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="A3" s="52" t="s">
+        <v>605</v>
+      </c>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="44"/>
@@ -6954,7 +6948,7 @@
     </row>
     <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="B5" s="30"/>
       <c r="C5" s="30"/>
@@ -6964,42 +6958,42 @@
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="32" t="s">
+        <v>607</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>608</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>609</v>
+      </c>
+      <c r="D6" s="29" t="s">
         <v>610</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="E6" s="29" t="s">
         <v>611</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="F6" s="29" t="s">
         <v>612</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="G6" s="29" t="s">
         <v>613</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="H6" s="29" t="s">
         <v>614</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="I6" s="29" t="s">
         <v>615</v>
-      </c>
-      <c r="G6" s="29" t="s">
-        <v>616</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>617</v>
-      </c>
-      <c r="I6" s="29" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D7" s="33" t="s">
         <v>220</v>
@@ -7012,13 +7006,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="D8" s="34"/>
       <c r="E8" s="34"/>
@@ -7032,10 +7026,10 @@
         <v>34</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>69</v>
@@ -7048,13 +7042,13 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="D10" s="33" t="s">
         <v>46</v>
@@ -7067,13 +7061,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>108</v>
@@ -7086,13 +7080,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="E12" s="42"/>
       <c r="F12" s="42"/>
@@ -7102,13 +7096,13 @@
     </row>
     <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="36" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="D13" s="33"/>
       <c r="E13" s="33"/>
@@ -7119,10 +7113,10 @@
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="37" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="C14" s="37"/>
       <c r="D14" s="34">
@@ -7136,10 +7130,10 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="D15" s="34"/>
       <c r="E15" s="43"/>
@@ -7149,14 +7143,14 @@
       <c r="I15" s="43"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="27" t="s">
-        <v>638</v>
+      <c r="A16" s="44" t="s">
+        <v>635</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33"/>
@@ -7167,10 +7161,10 @@
     </row>
     <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="37" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="C17" s="37"/>
       <c r="D17" s="34"/>
@@ -7182,13 +7176,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="E18" s="43"/>
       <c r="F18" s="43"/>
@@ -7198,13 +7192,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>644</v>
-      </c>
-      <c r="D19" s="52" t="s">
-        <v>645</v>
+        <v>641</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>642</v>
       </c>
       <c r="E19" s="43"/>
       <c r="F19" s="43"/>
@@ -7214,15 +7208,15 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>647</v>
-      </c>
-      <c r="D20" s="55" t="s">
+        <v>644</v>
+      </c>
+      <c r="D20" s="54" t="s">
         <v>108</v>
       </c>
       <c r="E20" s="33"/>
@@ -7314,46 +7308,46 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>581</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>
@@ -7380,52 +7374,52 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>581</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="I1" s="9" t="s">
         <v>660</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>589</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>661</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>662</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="E2" s="14"/>
       <c r="F2" s="8" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -7436,20 +7430,20 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="8" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -7460,22 +7454,22 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>668</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>669</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>670</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>671</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="F4" s="20" t="s">
         <v>672</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>673</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>674</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>675</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -7486,20 +7480,20 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="8" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -7510,20 +7504,20 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="8" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -7534,22 +7528,22 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B7" s="20" t="s">
+        <v>677</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>678</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>670</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>679</v>
+      </c>
+      <c r="F7" s="20" t="s">
         <v>680</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>681</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>673</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>682</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>683</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -7560,19 +7554,19 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B8" s="20" t="s">
+        <v>681</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>682</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>683</v>
+      </c>
+      <c r="F8" s="20" t="s">
         <v>684</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>685</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>686</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>687</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -7583,22 +7577,22 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B9" s="20" t="s">
+        <v>685</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>686</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>633</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>687</v>
+      </c>
+      <c r="F9" s="20" t="s">
         <v>688</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>689</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>636</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>690</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>691</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -7657,49 +7651,49 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>581</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>46</v>
@@ -7707,167 +7701,167 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
+        <v>707</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>710</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>708</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>713</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="15" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>